<commit_message>
reframe f01 panel g as a classification display, drop the circular t-test
</commit_message>
<xml_diff>
--- a/04_Figures/F01/c_data/F01_source_data.xlsx
+++ b/04_Figures/F01/c_data/F01_source_data.xlsx
@@ -703,9 +703,6 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -723,9 +720,6 @@
       <c r="E2" t="n">
         <v>1.39301445998033</v>
       </c>
-      <c r="F2" t="n">
-        <v>0.000000759141810025732</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
@@ -742,9 +736,6 @@
       </c>
       <c r="E3" t="n">
         <v>1.04120980457488</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.000000759141810025732</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
share one prepost-delta builder across the f01 panels and seed all jitter
</commit_message>
<xml_diff>
--- a/04_Figures/F01/c_data/F01_source_data.xlsx
+++ b/04_Figures/F01/c_data/F01_source_data.xlsx
@@ -7,10 +7,14 @@
   </bookViews>
   <sheets>
     <sheet name="panel_A_volume_load" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="panel_F_fiber_counts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="panel_G_hypertrophy_composite" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="panel_H_1rm_ext" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="panel_I_mcsa" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="panel_B_1rm_leg" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="panel_C_fcsa_mixed" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="panel_D_fcsa_type1" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="panel_E_fcsa_type2" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="panel_F_fiber_counts" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="panel_G_hypertrophy_composite" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="panel_H_1rm_ext" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="panel_I_mcsa" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
 </workbook>
 </file>
@@ -42,6 +46,18 @@
     <t xml:space="preserve">LR</t>
   </si>
   <si>
+    <t xml:space="preserve">delta_mean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">delta_sd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">delta_sem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">delta_t_test_p</t>
+  </si>
+  <si>
     <t xml:space="preserve">fiber_type</t>
   </si>
   <si>
@@ -58,18 +74,6 @@
   </si>
   <si>
     <t xml:space="preserve">Type_I</t>
-  </si>
-  <si>
-    <t xml:space="preserve">delta_mean</t>
-  </si>
-  <si>
-    <t xml:space="preserve">delta_sd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">delta_sem</t>
-  </si>
-  <si>
-    <t xml:space="preserve">delta_t_test_p</t>
   </si>
 </sst>
 </file>
@@ -471,209 +475,62 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
         <v>9</v>
       </c>
-      <c r="D1" t="s">
-        <v>1</v>
-      </c>
       <c r="E1" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="F1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
-        <v>11</v>
+      <c r="B2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" t="n">
+        <v>45</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>33.4108622200283</v>
       </c>
       <c r="E2" t="n">
-        <v>541.875</v>
+        <v>11.8125236205357</v>
       </c>
       <c r="F2" t="n">
-        <v>328.600251065029</v>
-      </c>
-      <c r="G2" t="n">
-        <v>116.177732913842</v>
+        <v>0.792860265103992</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
+        <v>7</v>
+      </c>
+      <c r="B3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3" t="n">
+        <v>40.625</v>
       </c>
       <c r="D3" t="n">
-        <v>8</v>
+        <v>31.9505756710937</v>
       </c>
       <c r="E3" t="n">
-        <v>395.5</v>
+        <v>11.2962343599221</v>
       </c>
       <c r="F3" t="n">
-        <v>156.962233856246</v>
-      </c>
-      <c r="G3" t="n">
-        <v>55.4945299749701</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" t="n">
-        <v>8</v>
-      </c>
-      <c r="E4" t="n">
-        <v>538.625</v>
-      </c>
-      <c r="F4" t="n">
-        <v>171.092237028535</v>
-      </c>
-      <c r="G4" t="n">
-        <v>60.4902405056268</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" t="n">
-        <v>8</v>
-      </c>
-      <c r="E5" t="n">
-        <v>753.375</v>
-      </c>
-      <c r="F5" t="n">
-        <v>190.129232365778</v>
-      </c>
-      <c r="G5" t="n">
-        <v>67.2208347538172</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" t="n">
-        <v>8</v>
-      </c>
-      <c r="E6" t="n">
-        <v>197.25</v>
-      </c>
-      <c r="F6" t="n">
-        <v>136.925162041168</v>
-      </c>
-      <c r="G6" t="n">
-        <v>48.4103552971882</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" t="n">
-        <v>8</v>
-      </c>
-      <c r="E7" t="n">
-        <v>154.125</v>
-      </c>
-      <c r="F7" t="n">
-        <v>84.3977614801314</v>
-      </c>
-      <c r="G7" t="n">
-        <v>29.8391147297828</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" t="n">
-        <v>8</v>
-      </c>
-      <c r="E8" t="n">
-        <v>188.5</v>
-      </c>
-      <c r="F8" t="n">
-        <v>88.6534182726677</v>
-      </c>
-      <c r="G8" t="n">
-        <v>31.3437166179854</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" t="n">
-        <v>8</v>
-      </c>
-      <c r="E9" t="n">
-        <v>263.25</v>
-      </c>
-      <c r="F9" t="n">
-        <v>77.3410813031655</v>
-      </c>
-      <c r="G9" t="n">
-        <v>27.3442015268842</v>
+        <v>0.792860265103992</v>
       </c>
     </row>
   </sheetData>
@@ -695,13 +552,16 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="2">
@@ -712,13 +572,16 @@
         <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>13.1</v>
+        <v>914.04625</v>
       </c>
       <c r="D2" t="n">
-        <v>3.94003988377203</v>
+        <v>883.987338951631</v>
       </c>
       <c r="E2" t="n">
-        <v>1.39301445998033</v>
+        <v>312.536720927875</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.00184410864144996</v>
       </c>
     </row>
     <row r="3">
@@ -729,13 +592,16 @@
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>-2.265</v>
+        <v>-961.9225</v>
       </c>
       <c r="D3" t="n">
-        <v>2.94498605381127</v>
+        <v>1055.1389135864</v>
       </c>
       <c r="E3" t="n">
-        <v>1.04120980457488</v>
+        <v>373.047940445374</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.00184410864144996</v>
       </c>
     </row>
   </sheetData>
@@ -757,16 +623,16 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="D1" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F1" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2">
@@ -774,19 +640,19 @@
         <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>10.7142857142857</v>
+        <v>889.5525</v>
       </c>
       <c r="D2" t="n">
-        <v>6.42168943799801</v>
+        <v>709.519588730894</v>
       </c>
       <c r="E2" t="n">
-        <v>2.42717046426184</v>
+        <v>250.853056288153</v>
       </c>
       <c r="F2" t="n">
-        <v>0.63242868562423</v>
+        <v>0.00111031808792228</v>
       </c>
     </row>
     <row r="3">
@@ -797,16 +663,16 @@
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>9</v>
+        <v>-1191.8375</v>
       </c>
       <c r="D3" t="n">
-        <v>7.13141941391353</v>
+        <v>1168.00511548232</v>
       </c>
       <c r="E3" t="n">
-        <v>2.52133751353183</v>
+        <v>412.952168809061</v>
       </c>
       <c r="F3" t="n">
-        <v>0.63242868562423</v>
+        <v>0.00111031808792228</v>
       </c>
     </row>
   </sheetData>
@@ -828,16 +694,438 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1043.16875</v>
+      </c>
+      <c r="D2" t="n">
+        <v>831.282904628013</v>
+      </c>
+      <c r="E2" t="n">
+        <v>293.902889473459</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.00104585273562438</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-870.95125</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1004.15080121659</v>
+      </c>
+      <c r="E3" t="n">
+        <v>355.020920437079</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.00104585273562438</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
         <v>14</v>
       </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2" t="n">
+        <v>541.875</v>
+      </c>
+      <c r="F2" t="n">
+        <v>328.600251065029</v>
+      </c>
+      <c r="G2" t="n">
+        <v>116.177732913842</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E3" t="n">
+        <v>395.5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>156.962233856246</v>
+      </c>
+      <c r="G3" t="n">
+        <v>55.4945299749701</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E4" t="n">
+        <v>538.625</v>
+      </c>
+      <c r="F4" t="n">
+        <v>171.092237028535</v>
+      </c>
+      <c r="G4" t="n">
+        <v>60.4902405056268</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" t="n">
+        <v>8</v>
+      </c>
+      <c r="E5" t="n">
+        <v>753.375</v>
+      </c>
+      <c r="F5" t="n">
+        <v>190.129232365778</v>
+      </c>
+      <c r="G5" t="n">
+        <v>67.2208347538172</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" t="n">
+        <v>197.25</v>
+      </c>
+      <c r="F6" t="n">
+        <v>136.925162041168</v>
+      </c>
+      <c r="G6" t="n">
+        <v>48.4103552971882</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" t="n">
+        <v>8</v>
+      </c>
+      <c r="E7" t="n">
+        <v>154.125</v>
+      </c>
+      <c r="F7" t="n">
+        <v>84.3977614801314</v>
+      </c>
+      <c r="G7" t="n">
+        <v>29.8391147297828</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" t="n">
+        <v>188.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>88.6534182726677</v>
+      </c>
+      <c r="G8" t="n">
+        <v>31.3437166179854</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" t="n">
+        <v>263.25</v>
+      </c>
+      <c r="F9" t="n">
+        <v>77.3410813031655</v>
+      </c>
+      <c r="G9" t="n">
+        <v>27.3442015268842</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
       <c r="D1" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>16</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>3.94003988377203</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.39301445998033</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-2.265</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2.94498605381127</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.04120980457488</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
+        <v>10</v>
       </c>
       <c r="F1" t="s">
-        <v>17</v>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2" t="n">
+        <v>10.7142857142857</v>
+      </c>
+      <c r="D2" t="n">
+        <v>6.42168943799801</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2.42717046426184</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.63242868562423</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D3" t="n">
+        <v>7.13141941391353</v>
+      </c>
+      <c r="E3" t="n">
+        <v>2.52133751353183</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.63242868562423</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="2">

</xml_diff>

<commit_message>
re-render figures and tables at the 1896-protein filtering baseline
</commit_message>
<xml_diff>
--- a/04_Figures/F01/c_data/F01_source_data.xlsx
+++ b/04_Figures/F01/c_data/F01_source_data.xlsx
@@ -6,21 +6,82 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="panel_A_volume_load" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="panel_B_1rm_leg" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="panel_C_fcsa_mixed" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="panel_D_fcsa_type1" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="panel_E_fcsa_type2" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="panel_F_myovision_fcsa" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="panel_G_hypertrophy_composite" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="panel_H_1rm_ext" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="panel_I_mcsa" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="panel_A_volume_load" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="panel_B_1rm_leg" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="panel_C_fcsa_mixed" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="panel_D_fcsa_type1" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="panel_E_fcsa_type2" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="panel_F_myovision_fcsa" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="panel_G_hypertrophy_composite" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="panel_H_1rm_ext" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="panel_I_mcsa" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+  <si>
+    <t xml:space="preserve">sheet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">panel_A_volume_load</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panel A: volume load</t>
+  </si>
+  <si>
+    <t xml:space="preserve">panel_B_1rm_leg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panel B: 1rm leg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">panel_C_fcsa_mixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panel C: fcsa mixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">panel_D_fcsa_type1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panel D: fcsa type1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">panel_E_fcsa_type2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panel E: fcsa type2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">panel_F_myovision_fcsa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panel F: myovision fcsa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">panel_G_hypertrophy_composite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panel G: hypertrophy composite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">panel_H_1rm_ext</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panel H: 1rm ext</t>
+  </si>
+  <si>
+    <t xml:space="preserve">panel_I_mcsa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panel I: mcsa</t>
+  </si>
   <si>
     <t xml:space="preserve">Group</t>
   </si>
@@ -409,57 +470,148 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="n">
-        <v>8</v>
-      </c>
-      <c r="C2" t="n">
-        <v>126078.625</v>
-      </c>
-      <c r="D2" t="n">
-        <v>51615.8804548077</v>
-      </c>
-      <c r="E2" t="n">
-        <v>18248.9695432544</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.642554614226018</v>
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
         <v>7</v>
       </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3.012625</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1.00774032050496</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.356290007152079</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.044028002060952</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
       <c r="B3" t="n">
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>139466.25</v>
+        <v>1.14125</v>
       </c>
       <c r="D3" t="n">
-        <v>60830.8359298849</v>
+        <v>2.0706159021619</v>
       </c>
       <c r="E3" t="n">
-        <v>21506.9482956339</v>
+        <v>0.732073272825689</v>
       </c>
       <c r="F3" t="n">
-        <v>0.642554614226018</v>
+        <v>0.044028002060952</v>
       </c>
     </row>
   </sheetData>
@@ -475,62 +627,62 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="E1" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F1" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="B2" t="n">
         <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>45</v>
+        <v>126078.625</v>
       </c>
       <c r="D2" t="n">
-        <v>33.4108622200283</v>
+        <v>51615.8804548077</v>
       </c>
       <c r="E2" t="n">
-        <v>11.8125236205357</v>
+        <v>18248.9695432544</v>
       </c>
       <c r="F2" t="n">
-        <v>0.792860265103992</v>
+        <v>0.642554614226018</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B3" t="n">
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>40.625</v>
+        <v>139466.25</v>
       </c>
       <c r="D3" t="n">
-        <v>31.9505756710937</v>
+        <v>60830.8359298849</v>
       </c>
       <c r="E3" t="n">
-        <v>11.2962343599221</v>
+        <v>21506.9482956339</v>
       </c>
       <c r="F3" t="n">
-        <v>0.792860265103992</v>
+        <v>0.642554614226018</v>
       </c>
     </row>
   </sheetData>
@@ -546,62 +698,62 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="E1" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F1" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="B2" t="n">
         <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>914.04625</v>
+        <v>45</v>
       </c>
       <c r="D2" t="n">
-        <v>883.987338951631</v>
+        <v>33.4108622200283</v>
       </c>
       <c r="E2" t="n">
-        <v>312.536720927875</v>
+        <v>11.8125236205357</v>
       </c>
       <c r="F2" t="n">
-        <v>0.00184410864144996</v>
+        <v>0.792860265103992</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B3" t="n">
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>-961.9225</v>
+        <v>40.625</v>
       </c>
       <c r="D3" t="n">
-        <v>1055.1389135864</v>
+        <v>31.9505756710937</v>
       </c>
       <c r="E3" t="n">
-        <v>373.047940445374</v>
+        <v>11.2962343599221</v>
       </c>
       <c r="F3" t="n">
-        <v>0.00184410864144996</v>
+        <v>0.792860265103992</v>
       </c>
     </row>
   </sheetData>
@@ -617,62 +769,62 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="E1" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F1" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="B2" t="n">
         <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>889.5525</v>
+        <v>914.04625</v>
       </c>
       <c r="D2" t="n">
-        <v>709.519588730894</v>
+        <v>883.987338951631</v>
       </c>
       <c r="E2" t="n">
-        <v>250.853056288153</v>
+        <v>312.536720927875</v>
       </c>
       <c r="F2" t="n">
-        <v>0.00111031808792228</v>
+        <v>0.00184410864144996</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B3" t="n">
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>-1191.8375</v>
+        <v>-961.9225</v>
       </c>
       <c r="D3" t="n">
-        <v>1168.00511548232</v>
+        <v>1055.1389135864</v>
       </c>
       <c r="E3" t="n">
-        <v>412.952168809061</v>
+        <v>373.047940445374</v>
       </c>
       <c r="F3" t="n">
-        <v>0.00111031808792228</v>
+        <v>0.00184410864144996</v>
       </c>
     </row>
   </sheetData>
@@ -688,62 +840,62 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="E1" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F1" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="B2" t="n">
         <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>1043.16875</v>
+        <v>889.5525</v>
       </c>
       <c r="D2" t="n">
-        <v>831.282904628013</v>
+        <v>709.519588730894</v>
       </c>
       <c r="E2" t="n">
-        <v>293.902889473459</v>
+        <v>250.853056288153</v>
       </c>
       <c r="F2" t="n">
-        <v>0.00104585273562438</v>
+        <v>0.00111031808792228</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B3" t="n">
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>-870.95125</v>
+        <v>-1191.8375</v>
       </c>
       <c r="D3" t="n">
-        <v>1004.15080121659</v>
+        <v>1168.00511548232</v>
       </c>
       <c r="E3" t="n">
-        <v>355.020920437079</v>
+        <v>412.952168809061</v>
       </c>
       <c r="F3" t="n">
-        <v>0.00104585273562438</v>
+        <v>0.00111031808792228</v>
       </c>
     </row>
   </sheetData>
@@ -759,209 +911,62 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="D1" t="s">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="E1" t="s">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="F1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" t="s">
-        <v>4</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>15</v>
+        <v>26</v>
+      </c>
+      <c r="B2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C2" t="n">
+        <v>1043.16875</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>831.282904628013</v>
       </c>
       <c r="E2" t="n">
-        <v>541.875</v>
+        <v>293.902889473459</v>
       </c>
       <c r="F2" t="n">
-        <v>328.600251065029</v>
-      </c>
-      <c r="G2" t="n">
-        <v>116.177732913842</v>
+        <v>0.00104585273562438</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" t="s">
-        <v>16</v>
+        <v>27</v>
+      </c>
+      <c r="B3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3" t="n">
+        <v>-870.95125</v>
       </c>
       <c r="D3" t="n">
-        <v>8</v>
+        <v>1004.15080121659</v>
       </c>
       <c r="E3" t="n">
-        <v>395.5</v>
+        <v>355.020920437079</v>
       </c>
       <c r="F3" t="n">
-        <v>156.962233856246</v>
-      </c>
-      <c r="G3" t="n">
-        <v>55.4945299749701</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" t="n">
-        <v>8</v>
-      </c>
-      <c r="E4" t="n">
-        <v>538.625</v>
-      </c>
-      <c r="F4" t="n">
-        <v>171.092237028535</v>
-      </c>
-      <c r="G4" t="n">
-        <v>60.4902405056268</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" t="n">
-        <v>8</v>
-      </c>
-      <c r="E5" t="n">
-        <v>753.375</v>
-      </c>
-      <c r="F5" t="n">
-        <v>190.129232365778</v>
-      </c>
-      <c r="G5" t="n">
-        <v>67.2208347538172</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" t="n">
-        <v>8</v>
-      </c>
-      <c r="E6" t="n">
-        <v>197.25</v>
-      </c>
-      <c r="F6" t="n">
-        <v>136.925162041168</v>
-      </c>
-      <c r="G6" t="n">
-        <v>48.4103552971882</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" t="n">
-        <v>8</v>
-      </c>
-      <c r="E7" t="n">
-        <v>154.125</v>
-      </c>
-      <c r="F7" t="n">
-        <v>84.3977614801314</v>
-      </c>
-      <c r="G7" t="n">
-        <v>29.8391147297828</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" t="n">
-        <v>8</v>
-      </c>
-      <c r="E8" t="n">
-        <v>188.5</v>
-      </c>
-      <c r="F8" t="n">
-        <v>88.6534182726677</v>
-      </c>
-      <c r="G8" t="n">
-        <v>31.3437166179854</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" t="n">
-        <v>8</v>
-      </c>
-      <c r="E9" t="n">
-        <v>263.25</v>
-      </c>
-      <c r="F9" t="n">
-        <v>77.3410813031655</v>
-      </c>
-      <c r="G9" t="n">
-        <v>27.3442015268842</v>
+        <v>0.00104585273562438</v>
       </c>
     </row>
   </sheetData>
@@ -977,53 +982,209 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>22</v>
+      </c>
+      <c r="F1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="n">
-        <v>8</v>
-      </c>
-      <c r="C2" t="n">
-        <v>13.1</v>
+        <v>34</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
       </c>
       <c r="D2" t="n">
-        <v>3.94003988377203</v>
+        <v>8</v>
       </c>
       <c r="E2" t="n">
-        <v>1.39301445998033</v>
+        <v>541.875</v>
+      </c>
+      <c r="F2" t="n">
+        <v>328.600251065029</v>
+      </c>
+      <c r="G2" t="n">
+        <v>116.177732913842</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="n">
-        <v>8</v>
-      </c>
-      <c r="C3" t="n">
-        <v>-2.265</v>
+        <v>34</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" t="s">
+        <v>36</v>
       </c>
       <c r="D3" t="n">
-        <v>2.94498605381127</v>
+        <v>8</v>
       </c>
       <c r="E3" t="n">
-        <v>1.04120980457488</v>
+        <v>395.5</v>
+      </c>
+      <c r="F3" t="n">
+        <v>156.962233856246</v>
+      </c>
+      <c r="G3" t="n">
+        <v>55.4945299749701</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4" t="n">
+        <v>8</v>
+      </c>
+      <c r="E4" t="n">
+        <v>538.625</v>
+      </c>
+      <c r="F4" t="n">
+        <v>171.092237028535</v>
+      </c>
+      <c r="G4" t="n">
+        <v>60.4902405056268</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" t="n">
+        <v>8</v>
+      </c>
+      <c r="E5" t="n">
+        <v>753.375</v>
+      </c>
+      <c r="F5" t="n">
+        <v>190.129232365778</v>
+      </c>
+      <c r="G5" t="n">
+        <v>67.2208347538172</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E6" t="n">
+        <v>197.25</v>
+      </c>
+      <c r="F6" t="n">
+        <v>136.925162041168</v>
+      </c>
+      <c r="G6" t="n">
+        <v>48.4103552971882</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" t="n">
+        <v>8</v>
+      </c>
+      <c r="E7" t="n">
+        <v>154.125</v>
+      </c>
+      <c r="F7" t="n">
+        <v>84.3977614801314</v>
+      </c>
+      <c r="G7" t="n">
+        <v>29.8391147297828</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" t="n">
+        <v>8</v>
+      </c>
+      <c r="E8" t="n">
+        <v>188.5</v>
+      </c>
+      <c r="F8" t="n">
+        <v>88.6534182726677</v>
+      </c>
+      <c r="G8" t="n">
+        <v>31.3437166179854</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" t="n">
+        <v>263.25</v>
+      </c>
+      <c r="F9" t="n">
+        <v>77.3410813031655</v>
+      </c>
+      <c r="G9" t="n">
+        <v>27.3442015268842</v>
       </c>
     </row>
   </sheetData>
@@ -1039,62 +1200,53 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="E1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F1" t="s">
-        <v>11</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="B2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>10.7142857142857</v>
+        <v>13.1</v>
       </c>
       <c r="D2" t="n">
-        <v>6.42168943799801</v>
+        <v>3.94003988377203</v>
       </c>
       <c r="E2" t="n">
-        <v>2.42717046426184</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.63242868562423</v>
+        <v>1.39301445998033</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B3" t="n">
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>9</v>
+        <v>-2.265</v>
       </c>
       <c r="D3" t="n">
-        <v>7.13141941391353</v>
+        <v>2.94498605381127</v>
       </c>
       <c r="E3" t="n">
-        <v>2.52133751353183</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.63242868562423</v>
+        <v>1.04120980457488</v>
       </c>
     </row>
   </sheetData>
@@ -1110,62 +1262,62 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="E1" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F1" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C2" t="n">
-        <v>3.012625</v>
+        <v>10.7142857142857</v>
       </c>
       <c r="D2" t="n">
-        <v>1.00774032050496</v>
+        <v>6.42168943799801</v>
       </c>
       <c r="E2" t="n">
-        <v>0.356290007152079</v>
+        <v>2.42717046426184</v>
       </c>
       <c r="F2" t="n">
-        <v>0.044028002060952</v>
+        <v>0.63242868562423</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B3" t="n">
         <v>8</v>
       </c>
       <c r="C3" t="n">
-        <v>1.14125</v>
+        <v>9</v>
       </c>
       <c r="D3" t="n">
-        <v>2.0706159021619</v>
+        <v>7.13141941391353</v>
       </c>
       <c r="E3" t="n">
-        <v>0.732073272825689</v>
+        <v>2.52133751353183</v>
       </c>
       <c r="F3" t="n">
-        <v>0.044028002060952</v>
+        <v>0.63242868562423</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
rebuild f01 on change scores: hedges g with holm, merged split panel, executable qmd
</commit_message>
<xml_diff>
--- a/04_Figures/F01/c_data/F01_source_data.xlsx
+++ b/04_Figures/F01/c_data/F01_source_data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="72">
   <si>
     <t xml:space="preserve">measure</t>
   </si>
@@ -35,16 +35,19 @@
     <t xml:space="preserve">delta_sem</t>
   </si>
   <si>
-    <t xml:space="preserve">lmm_advantage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lmm_ci_lo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lmm_ci_hi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lmm_p</t>
+    <t xml:space="preserve">g_advantage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g_ci_lo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g_ci_hi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p</t>
+  </si>
+  <si>
+    <t xml:space="preserve">p_holm</t>
   </si>
   <si>
     <t xml:space="preserve">icc</t>
@@ -200,22 +203,28 @@
     <t xml:space="preserve">HR/LR defined by the composite hypertrophy score; split is descriptive</t>
   </si>
   <si>
-    <t xml:space="preserve">model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lmer(value ~ Group*Timepoint + (1|subject)), REML, Satterthwaite df</t>
-  </si>
-  <si>
     <t xml:space="preserve">divergence</t>
   </si>
   <si>
-    <t xml:space="preserve">Group x Timepoint interaction; standardized as HR-minus-LR change advantage</t>
+    <t xml:space="preserve">per-subject change (T2-T1); HR-minus-LR standardized difference (Hedges g, SD units) with 95% CI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">two-sample t-test per outcome, Holm-adjusted across the six outcomes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">robustness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">the Group x Timepoint mixed model agrees at two timepoints; see the hlm supplement</t>
   </si>
   <si>
     <t xml:space="preserve">control</t>
   </si>
   <si>
-    <t xml:space="preserve">accumulated volume load compared by effect size + TOST equivalence</t>
+    <t xml:space="preserve">accumulated volume load: t-test with HR-LR difference + 95% CI, no equivalence claim at n=8/group</t>
   </si>
   <si>
     <t xml:space="preserve">source</t>
@@ -584,16 +593,19 @@
       <c r="K1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D2" t="n">
         <v>7</v>
@@ -605,30 +617,33 @@
         <v>2.42717046426184</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0651275774627513</v>
+        <v>0.236768258115466</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.232058767863854</v>
+        <v>-0.726452076278915</v>
       </c>
       <c r="I2" t="n">
-        <v>0.362313922789356</v>
+        <v>1.19105689676482</v>
       </c>
       <c r="J2" t="n">
-        <v>0.643809277651276</v>
+        <v>0.63242868562423</v>
       </c>
       <c r="K2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" t="n">
         <v>0.966109377270761</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D3" t="n">
         <v>8</v>
@@ -640,30 +655,33 @@
         <v>2.52133751353183</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0651275774627513</v>
+        <v>0.236768258115466</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.232058767863854</v>
+        <v>-0.726452076278915</v>
       </c>
       <c r="I3" t="n">
-        <v>0.362313922789356</v>
+        <v>1.19105689676482</v>
       </c>
       <c r="J3" t="n">
-        <v>0.643809277651276</v>
+        <v>0.63242868562423</v>
       </c>
       <c r="K3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" t="n">
         <v>0.966109377270761</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D4" t="n">
         <v>8</v>
@@ -675,30 +693,33 @@
         <v>11.8125236205357</v>
       </c>
       <c r="G4" t="n">
-        <v>0.082413492584948</v>
+        <v>0.126515027209886</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.577936733489977</v>
+        <v>-0.803244230735317</v>
       </c>
       <c r="I4" t="n">
-        <v>0.742763718659873</v>
+        <v>1.05181090559389</v>
       </c>
       <c r="J4" t="n">
-        <v>0.792852562803674</v>
+        <v>0.792860265103992</v>
       </c>
       <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="n">
         <v>0.788563846384003</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" t="s">
         <v>15</v>
-      </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
-        <v>14</v>
       </c>
       <c r="D5" t="n">
         <v>8</v>
@@ -710,30 +731,33 @@
         <v>11.2962343599221</v>
       </c>
       <c r="G5" t="n">
-        <v>0.082413492584948</v>
+        <v>0.126515027209886</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.577936733489977</v>
+        <v>-0.803244230735317</v>
       </c>
       <c r="I5" t="n">
-        <v>0.742763718659873</v>
+        <v>1.05181090559389</v>
       </c>
       <c r="J5" t="n">
-        <v>0.792852562803674</v>
+        <v>0.792860265103992</v>
       </c>
       <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
         <v>0.788563846384003</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D6" t="n">
         <v>8</v>
@@ -745,30 +769,33 @@
         <v>312.536720927875</v>
       </c>
       <c r="G6" t="n">
-        <v>1.27811582827483</v>
+        <v>1.82191646336275</v>
       </c>
       <c r="H6" t="n">
-        <v>0.566968013950189</v>
+        <v>0.658343657994327</v>
       </c>
       <c r="I6" t="n">
-        <v>1.98926364259948</v>
+        <v>2.94296960424087</v>
       </c>
       <c r="J6" t="n">
-        <v>0.0017511275799886</v>
+        <v>0.00184410864144996</v>
       </c>
       <c r="K6" t="n">
+        <v>0.00737643456579985</v>
+      </c>
+      <c r="L6" t="n">
         <v>0.777384858020191</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D7" t="n">
         <v>8</v>
@@ -780,30 +807,33 @@
         <v>373.047940445374</v>
       </c>
       <c r="G7" t="n">
-        <v>1.27811582827483</v>
+        <v>1.82191646336275</v>
       </c>
       <c r="H7" t="n">
-        <v>0.566968013950189</v>
+        <v>0.658343657994327</v>
       </c>
       <c r="I7" t="n">
-        <v>1.98926364259948</v>
+        <v>2.94296960424087</v>
       </c>
       <c r="J7" t="n">
-        <v>0.0017511275799886</v>
+        <v>0.00184410864144996</v>
       </c>
       <c r="K7" t="n">
+        <v>0.00737643456579985</v>
+      </c>
+      <c r="L7" t="n">
         <v>0.777384858020191</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" t="s">
         <v>18</v>
       </c>
-      <c r="B8" t="s">
-        <v>17</v>
-      </c>
       <c r="C8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D8" t="n">
         <v>8</v>
@@ -815,30 +845,33 @@
         <v>250.853056288153</v>
       </c>
       <c r="G8" t="n">
-        <v>1.56221016480904</v>
+        <v>2.03603046077722</v>
       </c>
       <c r="H8" t="n">
-        <v>0.784400533026606</v>
+        <v>0.824198483028628</v>
       </c>
       <c r="I8" t="n">
-        <v>2.34001979659148</v>
+        <v>3.20405353254597</v>
       </c>
       <c r="J8" t="n">
-        <v>0.000722632852588257</v>
+        <v>0.00111031808792229</v>
       </c>
       <c r="K8" t="n">
+        <v>0.00627511641374633</v>
+      </c>
+      <c r="L8" t="n">
         <v>0.714174618454065</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
         <v>18</v>
       </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
       <c r="C9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D9" t="n">
         <v>8</v>
@@ -850,30 +883,33 @@
         <v>412.952168809061</v>
       </c>
       <c r="G9" t="n">
-        <v>1.56221016480904</v>
+        <v>2.03603046077722</v>
       </c>
       <c r="H9" t="n">
-        <v>0.784400533026606</v>
+        <v>0.824198483028628</v>
       </c>
       <c r="I9" t="n">
-        <v>2.34001979659148</v>
+        <v>3.20405353254597</v>
       </c>
       <c r="J9" t="n">
-        <v>0.000722632852588257</v>
+        <v>0.00111031808792229</v>
       </c>
       <c r="K9" t="n">
+        <v>0.00627511641374633</v>
+      </c>
+      <c r="L9" t="n">
         <v>0.714174618454065</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D10" t="n">
         <v>8</v>
@@ -885,30 +921,33 @@
         <v>293.902889473459</v>
       </c>
       <c r="G10" t="n">
-        <v>1.10725736686667</v>
+        <v>1.96293875130603</v>
       </c>
       <c r="H10" t="n">
-        <v>0.53543655739102</v>
+        <v>0.767918548027783</v>
       </c>
       <c r="I10" t="n">
-        <v>1.67907817634232</v>
+        <v>3.11452350904239</v>
       </c>
       <c r="J10" t="n">
-        <v>0.000975649611071675</v>
+        <v>0.00104585273562439</v>
       </c>
       <c r="K10" t="n">
+        <v>0.00627511641374633</v>
+      </c>
+      <c r="L10" t="n">
         <v>0.858990196497898</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C11" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D11" t="n">
         <v>8</v>
@@ -920,30 +959,33 @@
         <v>355.020920437079</v>
       </c>
       <c r="G11" t="n">
-        <v>1.10725736686667</v>
+        <v>1.96293875130603</v>
       </c>
       <c r="H11" t="n">
-        <v>0.53543655739102</v>
+        <v>0.767918548027783</v>
       </c>
       <c r="I11" t="n">
-        <v>1.67907817634232</v>
+        <v>3.11452350904239</v>
       </c>
       <c r="J11" t="n">
-        <v>0.000975649611071675</v>
+        <v>0.00104585273562439</v>
       </c>
       <c r="K11" t="n">
+        <v>0.00627511641374633</v>
+      </c>
+      <c r="L11" t="n">
         <v>0.858990196497898</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D12" t="n">
         <v>8</v>
@@ -955,30 +997,33 @@
         <v>0.356290007152079</v>
       </c>
       <c r="G12" t="n">
-        <v>0.341871818128005</v>
+        <v>1.08637410733154</v>
       </c>
       <c r="H12" t="n">
-        <v>0.0228634869720242</v>
+        <v>0.0616415248383686</v>
       </c>
       <c r="I12" t="n">
-        <v>0.660880149283987</v>
+        <v>2.07863535710005</v>
       </c>
       <c r="J12" t="n">
-        <v>0.0374563196771928</v>
+        <v>0.044028002060952</v>
       </c>
       <c r="K12" t="n">
+        <v>0.132084006182856</v>
+      </c>
+      <c r="L12" t="n">
         <v>0.958156168084464</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C13" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D13" t="n">
         <v>8</v>
@@ -990,18 +1035,21 @@
         <v>0.732073272825689</v>
       </c>
       <c r="G13" t="n">
-        <v>0.341871818128005</v>
+        <v>1.08637410733154</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0228634869720242</v>
+        <v>0.0616415248383686</v>
       </c>
       <c r="I13" t="n">
-        <v>0.660880149283987</v>
+        <v>2.07863535710005</v>
       </c>
       <c r="J13" t="n">
-        <v>0.0374563196771928</v>
+        <v>0.044028002060952</v>
       </c>
       <c r="K13" t="n">
+        <v>0.132084006182856</v>
+      </c>
+      <c r="L13" t="n">
         <v>0.958156168084464</v>
       </c>
     </row>
@@ -1027,21 +1075,21 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" t="n">
         <v>8</v>
@@ -1058,10 +1106,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3" t="n">
         <v>8</v>
@@ -1078,10 +1126,10 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C4" t="n">
         <v>8</v>
@@ -1098,10 +1146,10 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C5" t="n">
         <v>8</v>
@@ -1118,27 +1166,27 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C8" t="n">
         <v>-6.6</v>
@@ -1152,10 +1200,10 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C9" t="n">
         <v>-5.99</v>
@@ -1169,10 +1217,10 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C10" t="n">
         <v>-4.09</v>
@@ -1186,10 +1234,10 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B11" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C11" t="n">
         <v>-1.86</v>
@@ -1203,10 +1251,10 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B12" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C12" t="n">
         <v>-0.74</v>
@@ -1220,10 +1268,10 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B13" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C13" t="n">
         <v>-0.48</v>
@@ -1237,10 +1285,10 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C14" t="n">
         <v>0.79</v>
@@ -1254,10 +1302,10 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B15" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C15" t="n">
         <v>0.85</v>
@@ -1271,10 +1319,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B16" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C16" t="n">
         <v>8.06</v>
@@ -1288,10 +1336,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B17" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C17" t="n">
         <v>9.43</v>
@@ -1305,10 +1353,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B18" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C18" t="n">
         <v>10.45</v>
@@ -1322,10 +1370,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B19" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C19" t="n">
         <v>13.69</v>
@@ -1339,10 +1387,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B20" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C20" t="n">
         <v>13.72</v>
@@ -1356,10 +1404,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B21" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C21" t="n">
         <v>13.79</v>
@@ -1373,10 +1421,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B22" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C22" t="n">
         <v>14.93</v>
@@ -1390,10 +1438,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B23" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C23" t="n">
         <v>20.73</v>
@@ -1421,27 +1469,27 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B2" t="n">
         <v>169.095339405363</v>
@@ -1464,7 +1512,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B3" t="n">
         <v>549.964052899636</v>
@@ -1487,7 +1535,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" t="n">
         <v>544.924733128971</v>
@@ -1510,7 +1558,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B5" t="n">
         <v>554.505196316068</v>
@@ -1533,7 +1581,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B6" t="n">
         <v>333.692499937065</v>
@@ -1556,7 +1604,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7" t="n">
         <v>257.432579175346</v>
@@ -1590,66 +1638,74 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B8" t="s">
-        <v>68</v>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>70</v>
+      </c>
+      <c r="B9" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>